<commit_message>
Update EnquireCTA message to focus on answering queries and questions
</commit_message>
<xml_diff>
--- a/public/registrations.xlsx
+++ b/public/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -763,9 +763,35 @@
         <v>3/4/2026, 12:51:33 am</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Krishna</v>
+      </c>
+      <c r="B15" t="str">
+        <v>7349975955</v>
+      </c>
+      <c r="C15" t="str">
+        <v>patil.tanisha1206@gmail.com</v>
+      </c>
+      <c r="D15" t="str">
+        <v>37 Prince city khatipura</v>
+      </c>
+      <c r="E15" t="str">
+        <v>10th Pass</v>
+      </c>
+      <c r="F15" t="str">
+        <v>WhatsApp</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Want to learn AI</v>
+      </c>
+      <c r="H15" t="str">
+        <v>3/4/2026, 2:18:17 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Add registration modal with progress tracker, update Google Sheets integration with AI Domain field
- Implement auto-popup registration modal with 15s delay and 30s close button reveal
- Add progress line animation that fills over 30 seconds
- Store custom AI Domain value when 'Others' is selected (instead of 'Other (Please Specify)')
- Remove OTP from Google Sheets (only used for email verification)
- Add AI Domain column to Google Sheets registration sheet
- Update excel.ts to match new data structure (remove otherAiDomain field)
- Implement body scroll lock hook for modal scrolling
- Add course details modals with learning objectives, tools, and enrollment flow
- Course cards now trigger registration modal via 'enrollNow' event
- Progress tracking: 15s auto-show, 30s close button reveal with visual progress bar
</commit_message>
<xml_diff>
--- a/public/registrations.xlsx
+++ b/public/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:J21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -789,9 +789,189 @@
         <v>3/4/2026, 2:18:17 pm</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Garv</v>
+      </c>
+      <c r="B16" t="str">
+        <v>6349975955</v>
+      </c>
+      <c r="C16" t="str">
+        <v>patil.tanisha1206@gmail.com</v>
+      </c>
+      <c r="D16" t="str">
+        <v>37 Prince city khatipura</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Post Graduate</v>
+      </c>
+      <c r="F16" t="str">
+        <v>WhatsApp</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Want to learn AI</v>
+      </c>
+      <c r="H16" t="str">
+        <v>3/4/2026, 3:36:04 pm</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>adarsh</v>
+      </c>
+      <c r="B17" t="str">
+        <v>5566778899</v>
+      </c>
+      <c r="C17" t="str">
+        <v>patil.tanisha1206@gmail.com</v>
+      </c>
+      <c r="D17" t="str">
+        <v>37 Prince city khatipura</v>
+      </c>
+      <c r="E17" t="str">
+        <v>12th Pass</v>
+      </c>
+      <c r="F17" t="str">
+        <v>AI Filmmaking &amp; Creative Design</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>Other</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Want to earn using AI</v>
+      </c>
+      <c r="J17" t="str">
+        <v>3/4/2026, 4:18:35 pm</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Ashish Bharti</v>
+      </c>
+      <c r="B18" t="str">
+        <v>7084896159</v>
+      </c>
+      <c r="C18" t="str">
+        <v>007lankanaresh@gmail.com</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Mirzapur</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Post Graduate</v>
+      </c>
+      <c r="F18" t="str">
+        <v>AI-Powered Digital Marketing</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>Friends</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Want to learn AI</v>
+      </c>
+      <c r="J18" t="str">
+        <v>3/4/2026, 5:59:03 pm</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>renee</v>
+      </c>
+      <c r="B19" t="str">
+        <v>8899007744</v>
+      </c>
+      <c r="C19" t="str">
+        <v>patil.tanisha1206@gmail.com</v>
+      </c>
+      <c r="D19" t="str">
+        <v>37 Prince city khatipura</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Graduate</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Other (Please Specify)</v>
+      </c>
+      <c r="G19" t="str">
+        <v>flim</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Facebook</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Want to learn AI</v>
+      </c>
+      <c r="J19" t="str">
+        <v>3/4/2026, 7:53:43 pm</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Tanisha patil</v>
+      </c>
+      <c r="B20" t="str">
+        <v>5349975955</v>
+      </c>
+      <c r="C20" t="str">
+        <v>shyammanohar1250@gmail.com</v>
+      </c>
+      <c r="D20" t="str">
+        <v>37 Prince city khatipura</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Graduate</v>
+      </c>
+      <c r="F20" t="str">
+        <v>SaaS Web Application Development</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Facebook</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Want to learn AI</v>
+      </c>
+      <c r="I20" t="str">
+        <v>4/4/2026, 8:51:47 am</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Tarun Singh</v>
+      </c>
+      <c r="B21" t="str">
+        <v>8858594654</v>
+      </c>
+      <c r="C21" t="str">
+        <v>shyammanohar1250@gmail.com</v>
+      </c>
+      <c r="D21" t="str">
+        <v>37 Prince city khatipura</v>
+      </c>
+      <c r="E21" t="str">
+        <v>10th Pass</v>
+      </c>
+      <c r="F21" t="str">
+        <v>flim</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Google</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Want to learn AI</v>
+      </c>
+      <c r="I21" t="str">
+        <v>4/4/2026, 8:55:17 am</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>